<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-10 Le livre d'Amir sous l'oreiller
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-10.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-10.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le nuage bateau d'Amir</t>
+          <t>Le livre d'Amir sous l'oreiller</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre à la lampe, classe, coin des livres</t>
+          <t>chambre à la lampe orange, classe, tapis, coin des livres</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amir, papa, maman, maîtresse</t>
+          <t>Amir, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut raconter le nuage en forme de bateau, puis montrer son livre. Il lève la main, il attend, puis il parle.</t>
+          <t>Un papillon de nuit tape le lampadaire. Sous l'oreiller, un livre a dormi. Sur une page, un éclat de page brille. Amir veut raconter le nuage bateau, maintenant. Il parle trop vite : les mots se perdent. Il ouvre trop vite : les pages claquent. Il refuse de foncer, lève la main, attend, puis dit. Merci vécu. Sous l'oreiller, l'éclat de page tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un papillon de nuit tape le lampadaire. Toc, toc, tout doux, contre l'abat-jour. La petite lampe orange fait un rond sur le mur. La croûte du pain a un peu de confiture. Amir, tes chaussures. Je fais le nœud. Le livre va dans le sac, tout à plat. Il est encore un peu chaud. Oui. Il a dormi près de l'oreiller. Tu as vu le nuage, par la fenêtre ? Il ressemblait à un bateau. Un bateau blanc, tout lent. Tu pourras le raconter. Le chemin sent le pain du fournil, au loin. On marche. Tu tiens ma manche. La classe sent les crayons et le papier. Au fond, le coin des livres a une petite lampe. La lumière est orange, comme à la maison. Au revoir, Amir. On revient. Au revoir, papa. Tu poses le sac près du tapis. En ce moment, Amir s'assoit sur le tapis. Le livre reste dans le sac, comme un secret. Il pose les mains sur ses genoux. Bonjour. Bonjour. Quelle forme avez-vous vue dans le ciel ? Amir a une idée. Le nuage bateau, blanc et lent. Le mot est déjà là. Il avance un peu sur le tapis. La maîtresse ouvre encore les volets. Un rectangle de lumière glisse sur le sol.</t>
+          <t>Un papillon de nuit tape le lampadaire. Toc, toc, contre l'abat-jour. La petite lampe orange fait un rond sur le mur. Amir connaît ce rond. La chambre sent le papier et la laine. Sous l'oreiller, un livre a dormi. Les pages sentent le papier, un peu chaud. Derrière la vitre, un nuage blanc passe. Sur une page, un éclat de page brille. Il est blanc, papa. C'est le bateau du livre. Le livre va dans le sac, à plat. Il a dormi sous l'oreiller. Tes chaussures, Amir. Je fais le nœud. Tu as vu le nuage, par la fenêtre ? Il ressemblait à un bateau. Un bateau blanc, dans le ciel. Je veux le raconter, maintenant ! Tu pourras le raconter. Papa parle près du sac, une main sur le tissu. Le nuage est un bateau ! Amir ouvre trop vite. Les pages claquent, puis se froissent. L'éclat de page saute près de l'oreiller. Les mots se cognent à ceux de papa. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le montrer ? Oui, papa. Tes pieds sont dans les chaussures ? Oui, maman. Tu tiens ma manche ? Oui. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent le pain du fournil. Le sac tape la hanche, un peu. On marche. La classe sent le papier et le bois. Au fond, le coin des livres a une lampe. La lumière est orange, comme à la maison. Au revoir, Amir. On revient. Au revoir, papa. Tu poses le sac près du tapis. En ce moment, Amir s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. Le livre reste dans le sac. Bonjour. Bonjour, maîtresse. Amir pose les mains sur ses genoux. Près du tapis, une image montre un ciel. Un camarade parle d'un oiseau. Je veux parler du bateau.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un papillon de nuit tape le lampadaire. Toc, toc, tout doux, contre l'abat-jour. La petite lampe orange fait un rond sur le mur. La croûte du pain a un peu de confiture. Amir, tes chaussures. Je fais le nœud. Le livre va dans le sac, tout à plat. Il est encore un peu chaud. Oui. Il a dormi près de l'oreiller. Tu as vu le nuage, par la fenêtre ? Il ressemblait à un bateau. Un bateau blanc, tout lent. Tu pourras le raconter. Le chemin sent le pain du fournil, au loin. On marche. Tu tiens ma manche. La classe sent les crayons et le papier. Au fond, le coin des livres a une petite lampe. La lumière est orange, comme à la maison. Au revoir, Amir. On revient. Au revoir, papa. Tu poses le sac près du tapis. En ce moment, Amir s'assoit sur le tapis. Le livre reste dans le sac, comme un secret. Il pose les mains sur ses genoux. Bonjour. Bonjour. Quelle forme avez-vous vue dans le ciel ? Amir a une idée. Le nuage bateau, blanc et lent. Le mot est déjà là. Il avance un peu sur le tapis. La maîtresse ouvre encore les volets. Un rectangle de lumière glisse sur le sol.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un papillon de nuit tape le lampadaire. Toc, toc, contre l'abat-jour. La petite lampe orange fait un rond sur le mur. Amir connaît ce rond. La chambre sent le papier et la laine. Sous l'oreiller, un livre a dormi. Les pages sentent le papier, un peu chaud. Derrière la vitre, un nuage blanc passe. Sur une page, un &lt;emphasis level="moderate"&gt;éclat de page&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le bateau du livre. Le livre va dans le sac, à plat. Il a dormi sous l'oreiller. Tes chaussures, Amir. Je fais le nœud. Tu as vu le nuage, par la fenêtre ? Il ressemblait à un bateau. Un bateau blanc, dans le ciel. Je veux le raconter, maintenant ! Tu pourras le raconter. Papa parle près du sac, une main sur le tissu. Le nuage est un bateau ! Amir ouvre trop vite. Les pages claquent, puis se froissent. L'éclat de page saute près de l'oreiller. Les mots se cognent à ceux de papa. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le montrer ? Oui, papa. Tes pieds sont dans les chaussures ? Oui, maman. Tu tiens ma manche ? Oui. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent le pain du fournil. Le sac tape la hanche, un peu. On marche. La classe sent le papier et le bois. Au fond, le coin des livres a une lampe. La lumière est orange, comme à la maison. Au revoir, Amir. On revient. Au revoir, papa. Tu poses le sac près du tapis. En ce moment, Amir s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. Le livre reste dans le sac. Bonjour. Bonjour, maîtresse. Amir pose les mains sur ses genoux. Près du tapis, une image montre un ciel. Un camarade parle d'un oiseau. Je veux parler du bateau.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Brice arrive en classe avec papa. Papa dit au revoir. Brice s'assoit sur le tapis. La maîtresse pose une question. Brice a une idée. Il lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Brice attend encore. Puis la maîtresse dit : Brice, c'est ton tour. Brice parle. Il dit : le nuage est blanc. La maîtresse sourit. Plus tard, au coin des livres, Brice a encore une idée. Même leçon, autre lieu. Il lève la main. Il attend. Puis parler, c'est son tour. Il dit : j'aime ce livre. Le soir, papa demande. Brice dit : j'ai levé la main. J'ai su attendre. Puis parler, c'était mon tour. [pause]</t>
+          <t>Un papillon de nuit tape le lampadaire. Toc, toc, contre l'abat-jour. La petite lampe orange fait un rond sur le mur. Amir connaît ce rond. La chambre sent le papier et la laine. Sous l'oreiller, un livre a dormi. Les pages sentent le papier, un peu chaud. Derrière la vitre, un nuage blanc passe. Sur une page, un &lt;emphasis&gt;éclat de page&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le bateau du livre. Le livre va dans le sac, à plat. Il a dormi sous l'oreiller. Tes chaussures, Amir. Je fais le nœud. Tu as vu le nuage, par la fenêtre ? Il ressemblait à un bateau. Un bateau blanc, dans le ciel. Je veux le raconter, maintenant ! Tu pourras le raconter. Papa parle près du sac, une main sur le tissu. Le nuage est un bateau ! Amir ouvre trop vite. Les pages claquent, puis se froissent. L'éclat de page saute près de l'oreiller. Les mots se cognent à ceux de papa. Oh. Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le montrer ? Oui, papa. Tes pieds sont dans les chaussures ? Oui, maman. Tu tiens ma manche ? Oui. On y va ? On y va. Au revoir, maman. Au revoir, Amir. Dehors, le chemin sent le pain du fournil. Le sac tape la hanche, un peu. On marche. La classe sent le papier et le bois. Au fond, le coin des livres a une lampe. La lumière est orange, comme à la maison. Au revoir, Amir. On revient. Au revoir, papa. Tu poses le sac près du tapis. En ce moment, Amir s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. Le livre reste dans le sac. Bonjour. Bonjour, maîtresse. Amir pose les mains sur ses genoux. Près du tapis, une image montre un ciel. Un camarade parle d'un oiseau. Je veux parler du bateau. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de page</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,45 +1326,74 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_raconter_le_bateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
           <t>narrateur|Un papillon de nuit tape le lampadaire.
-narrateur|Toc, toc, tout doux, contre l'abat-jour.
+narrateur|Toc, toc, contre l'abat-jour.
 narrateur|La petite lampe orange fait un rond sur le mur.
-narrateur|La croûte du pain a un peu de confiture.
-papa|Amir, tes chaussures.
+narrateur|Amir connaît ce rond.
+narrateur|La chambre sent le papier et la laine.
+narrateur|Sous l'oreiller, un livre a dormi.
+narrateur|Les pages sentent le papier, un peu chaud.
+narrateur|Derrière la vitre, un nuage blanc passe.
+narrateur|Sur une page, un éclat de page brille.
+enfant-m|Il est blanc, papa.
+papa|C'est le bateau du livre.
+maman|Le livre va dans le sac, à plat.
+enfant-m|Il a dormi sous l'oreiller.
+papa|Tes chaussures, Amir.
 papa|Je fais le nœud.
-maman|Le livre va dans le sac, tout à plat.
-enfant-m|Il est encore un peu chaud.
-papa|Oui.
-papa|Il a dormi près de l'oreiller.
 maman|Tu as vu le nuage, par la fenêtre ?
 enfant-m|Il ressemblait à un bateau.
-enfant-m|Un bateau blanc, tout lent.
+enfant-m|Un bateau blanc, dans le ciel.
+enfant-m|Je veux le raconter, maintenant !
 papa|Tu pourras le raconter.
-narrateur|Le chemin sent le pain du fournil, au loin.
+narrateur|Papa parle près du sac, une main sur le tissu.
+enfant-m|Le nuage est un bateau !
+narrateur|Amir ouvre trop vite.
+narrateur|Les pages claquent, puis se froissent.
+narrateur|L'éclat de page saute près de l'oreiller.
+narrateur|Les mots se cognent à ceux de papa.
+enfant-m|Oh.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le montrer ?
+enfant-m|Oui, papa.
+maman|Tes pieds sont dans les chaussures ?
+enfant-m|Oui, maman.
+papa|Tu tiens ma manche ?
+enfant-m|Oui.
+maman|On y va ?
+enfant-m|On y va.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Amir.
+narrateur|Dehors, le chemin sent le pain du fournil.
+narrateur|Le sac tape la hanche, un peu.
 maman|On marche.
-maman|Tu tiens ma manche.
-narrateur|La classe sent les crayons et le papier.
-narrateur|Au fond, le coin des livres a une petite lampe.
+narrateur|La classe sent le papier et le bois.
+narrateur|Au fond, le coin des livres a une lampe.
 narrateur|La lumière est orange, comme à la maison.
 papa|Au revoir, Amir.
 papa|On revient.
 enfant-m|Au revoir, papa.
 maman|Tu poses le sac près du tapis.
 narrateur|En ce moment, Amir s'assoit sur le tapis.
-narrateur|Le livre reste dans le sac, comme un secret.
-narrateur|Il pose les mains sur ses genoux.
+narrateur|Le tapis est un peu froid, sous les genoux.
+narrateur|Le livre reste dans le sac.
 maitresse|Bonjour.
-enfant-m|Bonjour.
-maitresse|Quelle forme avez-vous vue dans le ciel ?
-narrateur|Amir a une idée.
-narrateur|Le nuage bateau, blanc et lent.
-narrateur|Le mot est déjà là.
-narrateur|Il avance un peu sur le tapis.
-narrateur|La maîtresse ouvre encore les volets.
-narrateur|Un rectangle de lumière glisse sur le sol.</t>
+enfant-m|Bonjour, maîtresse.
+narrateur|Amir pose les mains sur ses genoux.
+narrateur|Près du tapis, une image montre un ciel.
+narrateur|Un camarade parle d'un oiseau.
+enfant-m|Je veux parler du bateau.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1401,12 +1430,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amir veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Amir veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Brice veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Amir veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-il d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1469,18 +1498,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1495,34 +1524,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1531,23 +1564,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_leve_la_main_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1580,17 +1613,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir lève la main. Il attend, la main haute. Il regarde la petite lampe orange, au fond. Sa main ne descend pas. Amir, c'est toi. Tu peux parler. Le nuage est blanc. Il ressemblait à un bateau. Il avançait tout doucement. Un bateau dans le ciel. Oui. Avec une voile, un peu. Merci, Amir. Plus tard, au coin des livres, la lampe est allumée. Amir ouvre son livre. Les pages sont un peu chaudes encore. Il a encore une idée. Il veut montrer le bateau du livre. Il lève la main. Il attend. Amir, c'est toi, ici aussi. J'aime ce livre. Il y a un bateau, aussi. Comme ton nuage. Comme mon nuage.</t>
+          <t>Amir ouvre la bouche trop vite. Le nuage est un bateau, maintenant ! Un camarade parle, près de l'image. J'ai vu un oiseau. Les deux voix se mélangent. Oh. Personne ne tourne la tête. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Amir attend que le silence arrive. Dans le sac, l'éclat de page brille. Je peux dire quelque chose ? Une tête se tourne vers lui. Le nuage est blanc. Il ressemblait au bateau du livre. Le livre a dormi sous l'oreiller. Les oreilles écoutent jusqu'au bout. Plus tard, au coin des livres, la lampe est allumée. Amir ouvre son livre. Les pages sont un peu chaudes. Je veux montrer le bateau. Il lève trop vite une page. La page se plie, presque. Oh. Amir refuse de foncer. Il referme la page. Il attend, les mains à plat. Amir. Le bateau est blanc. Comme le rond de la lampe. Le soir, la porte s'ouvre. Te voilà, Amir. Le sac est rentré. Amir pose le sac près de l'oreiller. Le nuage était un bateau. Comme dans le livre. Merci, Amir. Papa a entendu toute la phrase. Tu veux de l'eau ? Oui, maman. Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir lève la main. Il attend, la main haute. Il regarde la petite lampe orange, au fond. Sa main ne descend pas. Amir, c'est toi. Tu peux parler. Le nuage est blanc. Il ressemblait à un bateau. Il avançait tout doucement. Un bateau dans le ciel. Oui. Avec une voile, un peu. Merci, Amir. Plus tard, au coin des livres, la lampe est allumée. Amir ouvre son livre. Les pages sont un peu chaudes encore. Il a encore une idée. Il veut montrer le bateau du livre. Il lève la main. Il attend. Amir, c'est toi, ici aussi. J'aime ce livre. Il y a un bateau, aussi. Comme ton nuage. Comme mon nuage.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir ouvre la bouche trop vite. Le nuage est un bateau, &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;tenant ! Un camarade parle, près de l'image. J'ai vu un oiseau. Les deux voix se mélangent. Oh. Personne ne tourne la tête. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Amir attend que le silence arrive. Dans le sac, l'éclat de page brille. Je peux dire quelque chose ? Une tête se tourne vers lui. Le nuage est blanc. Il ressemblait au bateau du livre. Le livre a dormi sous l'oreiller. Les oreilles écoutent jusqu'au bout. Plus tard, au coin des livres, la lampe est allumée. Amir ouvre son livre. Les pages sont un peu chaudes. Je veux montrer le bateau. Il lève trop vite une page. La page se plie, presque. Oh. Amir refuse de foncer. Il referme la page. Il attend, les mains à plat. Amir. Le bateau est blanc. Comme le rond de la lampe. Le soir, la porte s'ouvre. Te voilà, Amir. Le sac est rentré. Amir pose le sac près de l'oreiller. Le nuage était un bateau. Comme dans le livre. Merci, Amir. Papa a entendu toute la phrase. Tu veux de l'eau ? Oui, maman. Le ventre d'Amir se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Brice a levé la main. Il a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; parler, c'était son tour. Au tapis, puis aux livres. [pause]</t>
+          <t>Amir ouvre la bouche trop vite. Le nuage est un bateau, &lt;emphasis&gt;main&lt;/emphasis&gt;tenant ! Un camarade parle, près de l'image. J'ai vu un oiseau. Les deux voix se mélangent. Oh. Personne ne tourne la tête. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Il lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Amir attend que le silence arrive. Dans le sac, l'éclat de page brille. Je peux dire quelque chose ? Une tête se tourne vers lui. Le nuage est blanc. Il ressemblait au bateau du livre. Le livre a dormi sous l'oreiller. Les oreilles écoutent jusqu'au bout. Plus tard, au coin des livres, la lampe est allumée. Amir ouvre son livre. Les pages sont un peu chaudes. Je veux montrer le bateau. Il lève trop vite une page. La page se plie, presque. Oh. Amir refuse de foncer. Il referme la page. Il attend, les mains à plat. Amir. Le bateau est blanc. Comme le rond de la lampe. Le soir, la porte s'ouvre. Te voilà, Amir. Le sac est rentré. Amir pose le sac près de l'oreiller. Le nuage était un bateau. Comme dans le livre. Merci, Amir. Papa a entendu toute la phrase. Tu veux de l'eau ? Oui, maman. Le ventre d'Amir se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1637,7 +1670,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1645,10 +1678,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1671,30 +1704,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>main</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1703,10 +1736,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1719,36 +1752,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_dit_le_nuage_bateau; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir lève la main.
-narrateur|Il attend, la main haute.
-narrateur|Il regarde la petite lampe orange, au fond.
-narrateur|Sa main ne descend pas.
-maitresse|Amir, c'est toi.
-maitresse|Tu peux parler.
+          <t>narrateur|Amir ouvre la bouche trop vite.
+enfant-m|Le nuage est un bateau, maintenant !
+narrateur|Un camarade parle, près de l'image.
+copain|J'ai vu un oiseau.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Personne ne tourne la tête.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il lève la main, près du tapis.
+narrateur|Sa main reste en l'air.
+narrateur|Le camarade finit sa phrase.
+narrateur|Amir attend que le silence arrive.
+narrateur|Dans le sac, l'éclat de page brille.
+enfant-m|Je peux dire quelque chose ?
+narrateur|Une tête se tourne vers lui.
 enfant-m|Le nuage est blanc.
-enfant-m|Il ressemblait à un bateau.
-enfant-m|Il avançait tout doucement.
-maitresse|Un bateau dans le ciel.
-enfant-m|Oui.
-enfant-m|Avec une voile, un peu.
-maitresse|Merci, Amir.
+enfant-m|Il ressemblait au bateau du livre.
+enfant-m|Le livre a dormi sous l'oreiller.
+narrateur|Les oreilles écoutent jusqu'au bout.
 narrateur|Plus tard, au coin des livres, la lampe est allumée.
 narrateur|Amir ouvre son livre.
-narrateur|Les pages sont un peu chaudes encore.
-narrateur|Il a encore une idée.
-narrateur|Il veut montrer le bateau du livre.
-narrateur|Il lève la main.
-narrateur|Il attend.
-maitresse|Amir, c'est toi, ici aussi.
-enfant-m|J'aime ce livre.
-enfant-m|Il y a un bateau, aussi.
-maitresse|Comme ton nuage.
-enfant-m|Comme mon nuage.</t>
+narrateur|Les pages sont un peu chaudes.
+enfant-m|Je veux montrer le bateau.
+narrateur|Il lève trop vite une page.
+narrateur|La page se plie, presque.
+enfant-m|Oh.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la page.
+narrateur|Il attend, les mains à plat.
+maitresse|Amir.
+enfant-m|Le bateau est blanc.
+enfant-m|Comme le rond de la lampe.
+narrateur|Le soir, la porte s'ouvre.
+papa|Te voilà, Amir.
+maman|Le sac est rentré.
+narrateur|Amir pose le sac près de l'oreiller.
+enfant-m|Le nuage était un bateau.
+enfant-m|Comme dans le livre.
+papa|Merci, Amir.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux de l'eau ?
+enfant-m|Oui, maman.
+narrateur|Le ventre d'Amir se desserre.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1780,17 +1833,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Amir range son cartable. Le livre glisse à plat, encore. La porte de l'école s'ouvre. Tu as passé un bon moment ? J'ai parlé du nuage bateau. Et du livre, aussi. Les deux bateaux ? Oui. Un dans le ciel. Un dans le livre. On rentre. Le pain du fournil sent encore. Le soir, la petite lampe orange se rallume. Le livre retrouve l'oreiller, tout près. Le papillon n'est plus là. Il est parti. Le bateau, lui, reste dans le livre.</t>
+          <t>Amir veut tout dire, d'un coup. Il saisit le livre trop vite. Les pages glissent vers le sol. Ça tombe ! Amir veut foncer, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le livre ouvert. Il écoute la chambre, un instant. La lampe orange tremble, un peu. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la page. Amir pose le livre, plus lentement. Il glisse le livre sous l'oreiller. L'oreiller est à sa place ? Oui, maman. Tes pieds sont près du lit ? Oui, papa. Il s'assoit au bord. Les pages se calment. Le papillon n'est plus là. Il est parti. Le bateau, lui, reste dans le livre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Amir range son cartable. Le livre glisse à plat, encore. La porte de l'école s'ouvre. Tu as passé un bon moment ? J'ai parlé du nuage bateau. Et du livre, aussi. Les deux bateaux ? Oui. Un dans le ciel. Un dans le livre. On rentre. Le pain du fournil sent encore. Le soir, la petite lampe orange se rallume. Le livre retrouve l'oreiller, tout près. Le papillon n'est plus là. Il est parti. Le bateau, lui, reste dans le livre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut tout dire, d'un coup. Il saisit le &lt;emphasis level="moderate"&gt;livre&lt;/emphasis&gt; trop vite. Les pages glissent vers le sol. Ça tombe ! Amir veut foncer, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le livre ouvert. Il écoute la chambre, un instant. La lampe orange tremble, un peu. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la page. Amir pose le livre, plus lentement. Il glisse le livre sous l'oreiller. L'oreiller est à sa place ? Oui, maman. Tes pieds sont près du lit ? Oui, papa. Il s'assoit au bord. Les pages se calment. Le papillon n'est plus là. Il est parti. Le bateau, lui, reste dans le livre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Brice range son cartable. Papa l'attend à la porte. [pause]</t>
+          <t>Amir veut tout dire, d'un coup. Il saisit le &lt;emphasis&gt;livre&lt;/emphasis&gt; trop vite. Les pages glissent vers le sol. Ça tombe ! Amir veut foncer, d'un coup. Amir refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le livre ouvert. Il écoute la chambre, un instant. La lampe orange tremble, un peu. Comme ce matin, papa ! Tu le vois, toi ? Oui, sur la page. Amir pose le livre, plus lentement. Il glisse le livre sous l'oreiller. L'oreiller est à sa place ? Oui, maman. Tes pieds sont près du lit ? Oui, papa. Il s'assoit au bord. Les pages se calment. Le papillon n'est plus là. Il est parti. Le bateau, lui, reste dans le livre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1837,7 +1890,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1845,10 +1898,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1869,28 +1922,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>livre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,10 +1956,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1913,26 +1970,39 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_couper_papa; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Amir range son cartable.
-narrateur|Le livre glisse à plat, encore.
-narrateur|La porte de l'école s'ouvre.
-papa|Tu as passé un bon moment ?
-enfant-m|J'ai parlé du nuage bateau.
-enfant-m|Et du livre, aussi.
-maman|Les deux bateaux ?
-enfant-m|Oui.
-enfant-m|Un dans le ciel.
-enfant-m|Un dans le livre.
-papa|On rentre.
-maman|Le pain du fournil sent encore.
-narrateur|Le soir, la petite lampe orange se rallume.
-narrateur|Le livre retrouve l'oreiller, tout près.
-enfant-m|Le papillon n'est plus là.
+          <t>narrateur|Amir veut tout dire, d'un coup.
+narrateur|Il saisit le livre trop vite.
+narrateur|Les pages glissent vers le sol.
+enfant-m|Ça tombe !
+narrateur|Amir veut foncer, d'un coup.
+narrateur|Amir refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde le livre ouvert.
+narrateur|Il écoute la chambre, un instant.
+narrateur|La lampe orange tremble, un peu.
+enfant-m|Comme ce matin, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur la page.
+narrateur|Amir pose le livre, plus lentement.
+narrateur|Il glisse le livre sous l'oreiller.
+maman|L'oreiller est à sa place ?
+enfant-m|Oui, maman.
+papa|Tes pieds sont près du lit ?
+enfant-m|Oui, papa.
+narrateur|Il s'assoit au bord.
+narrateur|Les pages se calment.
+narrateur|Le papillon n'est plus là.
 papa|Il est parti.
-maman|Le bateau, lui, reste dans le livre.</t>
+enfant-m|Le bateau, lui, reste dans le livre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1964,17 +2034,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les pages sentent encore le papier. Le nuage était un bateau. Bonne soirée, mon grand.</t>
+          <t>Ils restent près du lit. Le livre repose sous l'oreiller. L'éclat est là, papa. Tu le vois sur la page ? Oui, papa. On est bien, ici. La lampe orange fait un rond, plus petit. Le sac sent le papier, un peu. On m'a entendu. On t'a entendu, Amir. Oui, maman. Amir pose la joue près des pages. Les pages sont tièdes, un peu. C'est chaud. Tu le sens sur tes joues ? Oui, il est tiède. Dehors, le fournil s'endort. L'éclat de page tient sur la page.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les pages sentent encore le papier. Le nuage était un bateau. Bonne soirée, mon grand.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du lit. Le livre repose sous l'oreiller. L'éclat est là, papa. Tu le vois sur la page ? Oui, papa. On est bien, ici. La lampe orange fait un rond, plus petit. Le sac sent le papier, un peu. On m'a entendu. On t'a entendu, Amir. Oui, maman. Amir pose la joue près des pages. Les pages sont tièdes, un peu. C'est chaud. Tu le sens sur tes joues ? Oui, il est tiède. Dehors, le fournil s'endort. L'&lt;emphasis level="moderate"&gt;éclat de page&lt;/emphasis&gt; tient sur la page.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du lit. Le livre repose sous l'oreiller. L'éclat est là, papa. Tu le vois sur la page ? Oui, papa. On est bien, ici. La lampe orange fait un rond, plus petit. Le sac sent le papier, un peu. On m'a entendu. On t'a entendu, Amir. Oui, maman. Amir pose la joue près des pages. Les pages sont tièdes, un peu. C'est chaud. Tu le sens sur tes joues ? Oui, il est tiède. Dehors, le fournil s'endort. L'&lt;emphasis&gt;éclat de page&lt;/emphasis&gt; tient sur la page.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2021,18 +2091,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2041,12 +2111,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2055,17 +2125,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de page</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2074,11 +2148,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2087,26 +2161,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sous_l_oreiller; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Les pages sentent encore le papier.
-papa|Le nuage était un bateau.
-maman|Bonne soirée, mon grand.</t>
+          <t>narrateur|Ils restent près du lit.
+narrateur|Le livre repose sous l'oreiller.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur la page ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|La lampe orange fait un rond, plus petit.
+narrateur|Le sac sent le papier, un peu.
+enfant-m|On m'a entendu.
+maman|On t'a entendu, Amir.
+enfant-m|Oui, maman.
+narrateur|Amir pose la joue près des pages.
+narrateur|Les pages sont tièdes, un peu.
+enfant-m|C'est chaud.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est tiède.
+narrateur|Dehors, le fournil s'endort.
+narrateur|L'éclat de page tient sur la page.</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2212,6 +2305,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>